<commit_message>
Enhance exponential increase interpolation figure in data_load_mode.py
Refactor the _build_exponential_increase_interp_fig function to include additional parameters for better customization, such as per_concentration_cut, x_range_mode, show_experimental_data, legend_on_lines, and cut_at_x_max. This update improves the flexibility of the figure generation process. Additionally, implement a new supplementary figure for low R² cases in enzyme mode, providing a visual representation of linear fits and expected values for excluded concentrations, enhancing data analysis capabilities.
</commit_message>
<xml_diff>
--- a/Michaelis-Menten_calibration_results.xlsx
+++ b/Michaelis-Menten_calibration_results.xlsx
@@ -10,8 +10,9 @@
     <sheet name="Experimental data" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Time–FLU Interpolated curves" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Normalization results" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Fit results" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Model simulation input" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Supplementary fit v0-E" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Fit results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Model simulation input" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48324,6 +48325,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Condition (for supplementary plot)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Full linear fit R² &lt; 0.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Full linear fit R²</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.4266178340599613</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Low-3 linear equation</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>v₀ = 20477.504804 * [E] + 10778.499649</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Low-3 linear fit R²</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.9646330322656383</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Const fit range</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3rd-5th concentration points (sorted by [E])</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Const fit equation</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>v₀ = 33660.847717</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Const fit CV(RMSE) %</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>7.425038185536086</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>[E] (μg/mL)</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>Experimental v0</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Expected v0 (Low-3 linear fit)</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Expected v0 at not-used [E]</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Residual (Exp - Expected)</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Used in Low-3 fit</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Used in Const fit (3rd-5th)</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>Const-fit y (mean of 3rd-5th)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="B11" t="n">
+        <v>15762.85727379415</v>
+      </c>
+      <c r="C11" t="n">
+        <v>17177.71990005191</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>-1414.862626257764</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="B12" t="n">
+        <v>25699.23409062195</v>
+      </c>
+      <c r="C12" t="n">
+        <v>23576.94015123531</v>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>2122.293939386647</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="B13" t="n">
+        <v>35667.94934047321</v>
+      </c>
+      <c r="C13" t="n">
+        <v>36375.38065360209</v>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>-707.4313131288727</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>33660.84771692822</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B14" t="n">
+        <v>30137.64634396669</v>
+      </c>
+      <c r="C14" t="n">
+        <v>61972.26165833565</v>
+      </c>
+      <c r="D14" t="n">
+        <v>61972.26165833565</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-31834.61531436896</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>33660.84771692822</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" t="n">
+        <v>35176.94746634475</v>
+      </c>
+      <c r="C15" t="n">
+        <v>113166.0236678028</v>
+      </c>
+      <c r="D15" t="n">
+        <v>113166.0236678028</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-77989.07620145803</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>33660.84771692822</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -48386,7 +48673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Update general_analysis_mode.py to improve experiment type handling and visualization for v₀ vs [S] and v₀ vs [E] fits. Introduce helper functions for better modularity and enhance user feedback with appropriate subheaders based on experiment type. Update Michaelis-Menten calibration results file for consistency.
</commit_message>
<xml_diff>
--- a/Michaelis-Menten_calibration_results.xlsx
+++ b/Michaelis-Menten_calibration_results.xlsx
@@ -48119,7 +48119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -48150,15 +48150,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Initial→Exponent (t=0.1τ)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Exponent→Plateau (t=3τ)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Exponent→Plateau (t=3τ_max)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>v0 (RFU/min)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>R²</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Equation</t>
         </is>
@@ -48183,12 +48198,21 @@
         <v>0.5714543085543325</v>
       </c>
       <c r="F2" t="n">
+        <v>0.05714543085543326</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1.714362925662998</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1.714362925662998</v>
+      </c>
+      <c r="I2" t="n">
         <v>15762.85727379415</v>
       </c>
-      <c r="G2" t="n">
+      <c r="J2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>F(t) = 1.0000(1 - e^(-1.7499*t)), τ = 0.5715</t>
         </is>
@@ -48213,12 +48237,21 @@
         <v>0.4248690574246121</v>
       </c>
       <c r="F3" t="n">
+        <v>0.04248690574246122</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.274607172273836</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.714362925662998</v>
+      </c>
+      <c r="I3" t="n">
         <v>25699.23409062195</v>
       </c>
-      <c r="G3" t="n">
+      <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>F(t) = 1.0000(1 - e^(-2.3537*t)), τ = 0.4249</t>
         </is>
@@ -48243,12 +48276,21 @@
         <v>0.3818912176759815</v>
       </c>
       <c r="F4" t="n">
+        <v>0.03818912176759815</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.145673653027945</v>
+      </c>
+      <c r="H4" t="n">
+        <v>1.714362925662998</v>
+      </c>
+      <c r="I4" t="n">
         <v>35667.94934047321</v>
       </c>
-      <c r="G4" t="n">
+      <c r="J4" t="n">
         <v>1</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>F(t) = 1.0000(1 - e^(-2.6185*t)), τ = 0.3819</t>
         </is>
@@ -48273,12 +48315,21 @@
         <v>0.4857964179222402</v>
       </c>
       <c r="F5" t="n">
+        <v>0.04857964179222402</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.457389253766721</v>
+      </c>
+      <c r="H5" t="n">
+        <v>1.714362925662998</v>
+      </c>
+      <c r="I5" t="n">
         <v>30137.64634396669</v>
       </c>
-      <c r="G5" t="n">
+      <c r="J5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>F(t) = 1.0000(1 - e^(-2.0585*t)), τ = 0.4858</t>
         </is>
@@ -48303,12 +48354,21 @@
         <v>0.4513145066360355</v>
       </c>
       <c r="F6" t="n">
+        <v>0.04513145066360355</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.353943519908106</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1.714362925662998</v>
+      </c>
+      <c r="I6" t="n">
         <v>35176.94746634475</v>
       </c>
-      <c r="G6" t="n">
+      <c r="J6" t="n">
         <v>1</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>F(t) = 1.0000(1 - e^(-2.2157*t)), τ = 0.4513</t>
         </is>

</xml_diff>